<commit_message>
fix: unicef budget totals, embed annex diagrams, fill git answer
</commit_message>
<xml_diff>
--- a/Galeon_UNICEF_BudgetProposal.xlsx
+++ b/Galeon_UNICEF_BudgetProposal.xlsx
@@ -1298,9 +1298,7 @@
           <t>Engineering rigor &amp; ERC-20 pool deployment (current production chain)</t>
         </is>
       </c>
-      <c r="C7" s="105" t="n">
-        <v>9000</v>
-      </c>
+      <c r="C7" s="105" t="n"/>
       <c r="D7" s="105" t="n"/>
     </row>
     <row r="8" ht="15.6" customHeight="1">
@@ -1352,9 +1350,7 @@
           <t>External security delta-audit kickoff (Galeon-specific contracts + stealth library)</t>
         </is>
       </c>
-      <c r="C11" s="105" t="n">
-        <v>5500</v>
-      </c>
+      <c r="C11" s="105" t="n"/>
       <c r="D11" s="105" t="n"/>
     </row>
     <row r="12" ht="15.6" customHeight="1">
@@ -1406,9 +1402,7 @@
           <t>Partner discovery, LOI, and operational model scoping</t>
         </is>
       </c>
-      <c r="C15" s="105" t="n">
-        <v>5500</v>
-      </c>
+      <c r="C15" s="105" t="n"/>
       <c r="D15" s="105" t="n"/>
     </row>
     <row r="16" ht="17.45" customHeight="1">
@@ -1460,9 +1454,7 @@
           <t>Beneficiary onboarding — embedded email-based wallet and gas-simplification options</t>
         </is>
       </c>
-      <c r="C19" s="105" t="n">
-        <v>9250</v>
-      </c>
+      <c r="C19" s="105" t="n"/>
       <c r="D19" s="105" t="n"/>
     </row>
     <row r="20" ht="15.6" customHeight="1">
@@ -1530,9 +1522,7 @@
           <t>Real ASP filtering — sanctions screening + blocklist (replaces hackathon auto-approve)</t>
         </is>
       </c>
-      <c r="C24" s="105" t="n">
-        <v>9000</v>
-      </c>
+      <c r="C24" s="105" t="n"/>
       <c r="D24" s="105" t="n"/>
     </row>
     <row r="25" ht="15.6" customHeight="1">
@@ -1584,9 +1574,7 @@
           <t>Audit findings remediated; final audit report published</t>
         </is>
       </c>
-      <c r="C28" s="105" t="n">
-        <v>21000</v>
-      </c>
+      <c r="C28" s="105" t="n"/>
       <c r="D28" s="105" t="n"/>
     </row>
     <row r="29">
@@ -1638,9 +1626,7 @@
           <t>Children's data protection — DPIA review and in-product safeguards</t>
         </is>
       </c>
-      <c r="C32" s="105" t="n">
-        <v>6500</v>
-      </c>
+      <c r="C32" s="105" t="n"/>
       <c r="D32" s="105" t="n"/>
     </row>
     <row r="33">
@@ -1692,9 +1678,7 @@
           <t>Open-source community readiness + sandbox with partner staff</t>
         </is>
       </c>
-      <c r="C36" s="105" t="n">
-        <v>7750</v>
-      </c>
+      <c r="C36" s="105" t="n"/>
       <c r="D36" s="105" t="n"/>
     </row>
     <row r="37">
@@ -1762,9 +1746,7 @@
           <t>Controlled pilot launch with LOI partner (≤50 beneficiaries)</t>
         </is>
       </c>
-      <c r="C41" s="105" t="n">
-        <v>7150</v>
-      </c>
+      <c r="C41" s="105" t="n"/>
       <c r="D41" s="105" t="n"/>
     </row>
     <row r="42" ht="17.85" customHeight="1">
@@ -1816,9 +1798,7 @@
           <t>Shipwreck jurisdiction expansion and multi-language UI (English + one pilot language)</t>
         </is>
       </c>
-      <c r="C45" s="105" t="n">
-        <v>5000</v>
-      </c>
+      <c r="C45" s="105" t="n"/>
       <c r="D45" s="105" t="n"/>
     </row>
     <row r="46">
@@ -1870,9 +1850,7 @@
           <t>Pilot validation and feedback</t>
         </is>
       </c>
-      <c r="C49" s="105" t="n">
-        <v>2500</v>
-      </c>
+      <c r="C49" s="105" t="n"/>
       <c r="D49" s="105" t="n"/>
     </row>
     <row r="50">
@@ -1988,9 +1966,7 @@
           <t>Pilot expansion to ≤100 beneficiaries</t>
         </is>
       </c>
-      <c r="C58" s="105" t="n">
-        <v>5100</v>
-      </c>
+      <c r="C58" s="105" t="n"/>
       <c r="D58" s="105" t="n"/>
     </row>
     <row r="59">
@@ -2042,9 +2018,7 @@
           <t>Implementation and usability evaluation co-conducted with partner M&amp;E lead</t>
         </is>
       </c>
-      <c r="C62" s="105" t="n">
-        <v>1500</v>
-      </c>
+      <c r="C62" s="105" t="n"/>
       <c r="D62" s="105" t="n"/>
     </row>
     <row r="63">
@@ -2096,9 +2070,7 @@
           <t>Developer documentation and integration guides</t>
         </is>
       </c>
-      <c r="C66" s="105" t="n">
-        <v>3000</v>
-      </c>
+      <c r="C66" s="105" t="n"/>
       <c r="D66" s="105" t="n"/>
     </row>
     <row r="67">
@@ -2150,9 +2122,7 @@
           <t>Sustainability roadmap, partner engagement, and final validation + accessibility conformance review</t>
         </is>
       </c>
-      <c r="C70" s="106" t="n">
-        <v>2250</v>
-      </c>
+      <c r="C70" s="106" t="n"/>
       <c r="D70" s="106" t="n"/>
     </row>
     <row r="71">

</xml_diff>